<commit_message>
feat: make Cuadrilla (CDLLA) field editable in form (v5.0)
</commit_message>
<xml_diff>
--- a/METRADO_PLANTILLA_3.xlsx
+++ b/METRADO_PLANTILLA_3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00_OFI_PRESUPUESTOS_progra\3_Entregable_web_buscador_de_metrados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E3DD2E5-A324-4270-864E-2E10D2AF347B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08A71EB5-05FE-4E29-BBEB-78F9296DDAD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2692,7 +2692,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="226">
   <si>
     <t>Item</t>
   </si>
@@ -3368,6 +3368,9 @@
   <si>
     <t>UNIDAD</t>
   </si>
+  <si>
+    <t>MODIF.</t>
+  </si>
 </sst>
 </file>
 
@@ -3964,7 +3967,43 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color rgb="FFFF0000"/>
+        <name val="Arial Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="hair">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="hair">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="hair">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="hair">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -4075,9 +4114,9 @@
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="METRADO-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="firstRowStripe" dxfId="4"/>
-      <tableStyleElement type="secondRowStripe" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="6"/>
+      <tableStyleElement type="firstRowStripe" dxfId="5"/>
+      <tableStyleElement type="secondRowStripe" dxfId="4"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -4414,15 +4453,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="B7:U419">
-  <tableColumns count="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="B7:V419">
+  <tableColumns count="21">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="GRADO"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="FECHA"/>
-    <tableColumn id="22" xr3:uid="{75338989-54C4-42C0-AB0F-AD00D70509B6}" name="ESPECIALIDAD" dataDxfId="2"/>
+    <tableColumn id="22" xr3:uid="{75338989-54C4-42C0-AB0F-AD00D70509B6}" name="ESPECIALIDAD" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="FRENTE"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="BLOQUE"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="NIVEL (PISO)"/>
-    <tableColumn id="20" xr3:uid="{27C08F62-596F-4FBA-9EF8-7774AD5B9C24}" name="CUADRILLA" dataDxfId="1"/>
+    <tableColumn id="20" xr3:uid="{27C08F62-596F-4FBA-9EF8-7774AD5B9C24}" name="CUADRILLA" dataDxfId="2"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="ITEM (CODIGO)"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="PARTIDA"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="DESCRIPCIÓN"/>
@@ -4434,8 +4473,9 @@
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="ACERO"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="N° VECES"/>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="TOTAL"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="TOTAL 2" dataDxfId="0"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="TOTAL 2" dataDxfId="1"/>
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="UNIDAD"/>
+    <tableColumn id="19" xr3:uid="{C63B1A4F-195F-49E5-8E64-665A403483B3}" name="MODIF." dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="METRADO-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -33003,7 +33043,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AL1000"/>
+  <dimension ref="A1:V1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.44140625" customWidth="1"/>
@@ -33249,7 +33289,7 @@
         <v>224</v>
       </c>
       <c r="V7" s="38" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
docs: update METRADO_PLANTILLA_3.xlsx with user aesthetic changes (v5.1)
</commit_message>
<xml_diff>
--- a/METRADO_PLANTILLA_3.xlsx
+++ b/METRADO_PLANTILLA_3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00_OFI_PRESUPUESTOS_progra\3_Entregable_web_buscador_de_metrados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08A71EB5-05FE-4E29-BBEB-78F9296DDAD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{048FFE1E-DA3E-4199-8311-9978C20DC2FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2692,7 +2692,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="225">
   <si>
     <t>Item</t>
   </si>
@@ -3349,9 +3349,6 @@
   </si>
   <si>
     <t>GRADO</t>
-  </si>
-  <si>
-    <t>NIVEL INDIC.</t>
   </si>
   <si>
     <t>TOTAL 2</t>
@@ -4214,7 +4211,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>403860</xdr:colOff>
+      <xdr:colOff>826531</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>91440</xdr:rowOff>
     </xdr:to>
@@ -4275,7 +4272,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>403860</xdr:colOff>
+      <xdr:colOff>826531</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>91440</xdr:rowOff>
     </xdr:to>
@@ -4336,7 +4333,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>403860</xdr:colOff>
+      <xdr:colOff>826531</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>91440</xdr:rowOff>
     </xdr:to>
@@ -4397,7 +4394,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>403860</xdr:colOff>
+      <xdr:colOff>826531</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>91440</xdr:rowOff>
     </xdr:to>
@@ -4470,8 +4467,8 @@
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="ANCHO / EMPAME"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="ALTURA / GANCHO"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="PARCIAL"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="ACERO"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="N° VECES"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="N° VECES"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="ACERO"/>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="TOTAL"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="TOTAL 2" dataDxfId="1"/>
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="UNIDAD"/>
@@ -33047,23 +33044,23 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.44140625" customWidth="1"/>
-    <col min="2" max="5" width="7.44140625" customWidth="1"/>
-    <col min="6" max="6" width="8.44140625" customWidth="1"/>
-    <col min="7" max="7" width="7.44140625" customWidth="1"/>
+    <col min="2" max="4" width="7.44140625" customWidth="1"/>
+    <col min="5" max="7" width="6.5546875" customWidth="1"/>
     <col min="8" max="8" width="9.33203125" customWidth="1"/>
-    <col min="9" max="9" width="11.44140625" customWidth="1"/>
-    <col min="10" max="10" width="31.77734375" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" customWidth="1"/>
+    <col min="10" max="10" width="38.21875" customWidth="1"/>
     <col min="11" max="11" width="38.88671875" customWidth="1"/>
     <col min="12" max="12" width="9.6640625" customWidth="1"/>
     <col min="13" max="13" width="13.44140625" customWidth="1"/>
     <col min="14" max="14" width="14.44140625" customWidth="1"/>
     <col min="15" max="15" width="15.109375" customWidth="1"/>
     <col min="16" max="16" width="7" customWidth="1"/>
-    <col min="17" max="17" width="9" customWidth="1"/>
-    <col min="18" max="18" width="5.6640625" customWidth="1"/>
-    <col min="19" max="19" width="10.109375" customWidth="1"/>
+    <col min="17" max="17" width="5.88671875" customWidth="1"/>
+    <col min="18" max="18" width="6.44140625" customWidth="1"/>
+    <col min="19" max="19" width="9.109375" customWidth="1"/>
     <col min="20" max="20" width="8" style="95" customWidth="1"/>
-    <col min="21" max="22" width="11.44140625" customWidth="1"/>
+    <col min="21" max="21" width="11.44140625" customWidth="1"/>
+    <col min="22" max="22" width="10.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -33202,9 +33199,7 @@
     </row>
     <row r="6" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="25"/>
-      <c r="B6" s="26" t="s">
-        <v>219</v>
-      </c>
+      <c r="B6" s="26"/>
       <c r="C6" s="27"/>
       <c r="D6" s="27"/>
       <c r="E6" s="27"/>
@@ -33243,14 +33238,14 @@
       <c r="F7" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="G7" s="40" t="s">
+      <c r="G7" s="42" t="s">
+        <v>220</v>
+      </c>
+      <c r="H7" s="40" t="s">
         <v>221</v>
       </c>
-      <c r="H7" s="40" t="s">
+      <c r="I7" s="42" t="s">
         <v>222</v>
-      </c>
-      <c r="I7" s="40" t="s">
-        <v>223</v>
       </c>
       <c r="J7" s="41" t="s">
         <v>17</v>
@@ -33274,22 +33269,22 @@
         <v>48</v>
       </c>
       <c r="Q7" s="42" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="R7" s="42" t="s">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="S7" s="40" t="s">
         <v>32</v>
       </c>
       <c r="T7" s="83" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="U7" s="38" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="V7" s="38" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>